<commit_message>
chore(S1): re-export Sprint 1 deliverables after DEF-F1-01 fix
Refs: P11

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018dPQXAbe9nEc4NmUbYrVzF
</commit_message>
<xml_diff>
--- a/deliverables/S1/HK261_SPM_FP_Team6_c2_SprintBacklog_S1.xlsx
+++ b/deliverables/S1/HK261_SPM_FP_Team6_c2_SprintBacklog_S1.xlsx
@@ -2264,7 +2264,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -2272,7 +2272,7 @@
     <col width="33" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="53" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
   </cols>
@@ -2336,122 +2336,102 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Hồ Du Tuấn Đạt (AI-assisted)</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Manual run found defect DEF-F1-01 (TC-F1-15); expected result made precise; E2E assertion tightened</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Version history</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>TC</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>AC</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Given</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>When (steps)</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>Then (expected)</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>Automated</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>Actual – local automated</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>Actual – hosted, manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>TC-F1-01</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>US-01/AC-01</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Register page open</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Submit valid name, new email, password Reader2026</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Account created as Customer, signed in, redirected home</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>E2E + INT</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>Pass (30/10)</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-02</t>
+          <t>TC-F1-01</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>US-01/AC-02</t>
+          <t>US-01/AC-01</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Customer x@y.com exists</t>
+          <t>Register page open</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Register with X@Y.COM</t>
+          <t>Submit valid name, new email, password Reader2026</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>"Email is already registered" by email field; no new account</t>
+          <t>Account created as Customer, signed in, redirected home</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -2473,27 +2453,27 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-03</t>
+          <t>TC-F1-02</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>US-01/AC-03</t>
+          <t>US-01/AC-02</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Register page open</t>
+          <t>Customer x@y.com exists</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Submit not-an-email; then empty fields; then POST bypassing client</t>
+          <t>Register with X@Y.COM</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Field errors on client; server also rejects</t>
+          <t>"Email is already registered" by email field; no new account</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -2515,12 +2495,12 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-04</t>
+          <t>TC-F1-03</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>US-01/AC-04</t>
+          <t>US-01/AC-03</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -2530,17 +2510,17 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Password abc1234 (7) then abcd1234 (8)</t>
+          <t>Submit not-an-email; then empty fields; then POST bypassing client</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>7 rejected, 8 accepted</t>
+          <t>Field errors on client; server also rejects</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>E2E + UNIT</t>
+          <t>E2E + INT</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -2557,32 +2537,32 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-05</t>
+          <t>TC-F1-04</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>US-02/AC-01</t>
+          <t>US-01/AC-04</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Active account</t>
+          <t>Register page open</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Log in with correct credentials</t>
+          <t>Password abc1234 (7) then abcd1234 (8)</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Signed in; name and Log out shown</t>
+          <t>7 rejected, 8 accepted</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>E2E + INT</t>
+          <t>E2E + UNIT</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -2599,12 +2579,12 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-06</t>
+          <t>TC-F1-05</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>US-02/AC-02</t>
+          <t>US-02/AC-01</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -2614,12 +2594,12 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Log in with wrong password; with unknown email</t>
+          <t>Log in with correct credentials</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Same generic "Invalid email or password"</t>
+          <t>Signed in; name and Log out shown</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -2641,27 +2621,27 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-07</t>
+          <t>TC-F1-06</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>US-02/AC-03</t>
+          <t>US-02/AC-02</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Account locked by admin</t>
+          <t>Active account</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Log in with correct credentials</t>
+          <t>Log in with wrong password; with unknown email</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>"This account is locked…"</t>
+          <t>Same generic "Invalid email or password"</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
@@ -2683,32 +2663,32 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-08</t>
+          <t>TC-F1-07</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>US-02/AC-04</t>
+          <t>US-02/AC-03</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Signed in</t>
+          <t>Account locked by admin</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Click Log out; open /admin</t>
+          <t>Log in with correct credentials</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Session ended; redirected to Login</t>
+          <t>"This account is locked…"</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>E2E</t>
+          <t>E2E + INT</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -2725,32 +2705,32 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-09</t>
+          <t>TC-F1-08</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>US-02/AC-05</t>
+          <t>US-02/AC-04</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Account e@x.com</t>
+          <t>Signed in</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Log in with   E@X.COM </t>
+          <t>Click Log out; open /admin</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Signed in</t>
+          <t>Session ended; redirected to Login</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>E2E + INT + UNIT</t>
+          <t>E2E</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -2767,32 +2747,32 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-10</t>
+          <t>TC-F1-09</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>US-03/AC-01</t>
+          <t>US-02/AC-05</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Signed in as admin</t>
+          <t>Account e@x.com</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Create account with role Customer</t>
+          <t xml:space="preserve">Log in with   E@X.COM </t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Appears in list, role Customer, Active</t>
+          <t>Signed in</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>E2E + INT</t>
+          <t>E2E + INT + UNIT</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -2809,27 +2789,27 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-11</t>
+          <t>TC-F1-10</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>US-03/AC-02</t>
+          <t>US-03/AC-01</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Admin; another active account</t>
+          <t>Signed in as admin</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Lock, then Unlock</t>
+          <t>Create account with role Customer</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Locked user cannot log in; after unlock can</t>
+          <t>Appears in list, role Customer, Active</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
@@ -2851,27 +2831,27 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-12</t>
+          <t>TC-F1-11</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>US-03/AC-03</t>
+          <t>US-03/AC-02</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Signed in as admin</t>
+          <t>Admin; another active account</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Click Lock on own row</t>
+          <t>Lock, then Unlock</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>"You cannot lock your own account"</t>
+          <t>Locked user cannot log in; after unlock can</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
@@ -2893,27 +2873,27 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-13</t>
+          <t>TC-F1-12</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>US-03/AC-04</t>
+          <t>US-03/AC-03</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Admin; email exists</t>
+          <t>Signed in as admin</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Create account with that email</t>
+          <t>Click Lock on own row</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Field error; no account</t>
+          <t>"You cannot lock your own account"</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
@@ -2935,27 +2915,27 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-14</t>
+          <t>TC-F1-13</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>US-03/AC-05</t>
+          <t>US-03/AC-04</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>User signed in in another browser</t>
+          <t>Admin; email exists</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Admin locks that user; user reloads</t>
+          <t>Create account with that email</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>User is signed out</t>
+          <t>Field error; no account</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
@@ -2977,32 +2957,32 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-15</t>
+          <t>TC-F1-14</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>US-04/AC-01</t>
+          <t>US-03/AC-05</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Not signed in</t>
+          <t>User signed in in another browser</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Open /admin/accounts</t>
+          <t>Admin locks that user; user reloads</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Redirect to /login?next=…</t>
+          <t>User is signed out</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>E2E</t>
+          <t>E2E + INT</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
@@ -3019,27 +2999,27 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-16</t>
+          <t>TC-F1-15</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>US-04/AC-02</t>
+          <t>US-04/AC-01</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Signed in as Customer</t>
+          <t>Not signed in</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Open /admin/accounts directly</t>
+          <t>Open /admin/accounts</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>HTTP 403 "Access denied"</t>
+          <t>Redirect to /login?next=%2Fadmin%2Faccounts; after login back on that page</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
@@ -3061,27 +3041,27 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-17</t>
+          <t>TC-F1-16</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>US-04/AC-03</t>
+          <t>US-04/AC-02</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Signed in as admin</t>
+          <t>Signed in as Customer</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Open /admin</t>
+          <t>Open /admin/accounts directly</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Admin dashboard shown</t>
+          <t>HTTP 403 "Access denied"</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
@@ -3103,27 +3083,27 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-18</t>
+          <t>TC-F1-17</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>US-04/AC-04</t>
+          <t>US-04/AC-03</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Signed in as Customer</t>
+          <t>Signed in as admin</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Look at header on any page</t>
+          <t>Open /admin</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>No Admin menu</t>
+          <t>Admin dashboard shown</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
@@ -3145,32 +3125,32 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-19</t>
+          <t>TC-F1-18</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>NFR-01/AC-01</t>
+          <t>US-04/AC-04</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>New account saved</t>
+          <t>Signed in as Customer</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Inspect users.password_hash in DB</t>
+          <t>Look at header on any page</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>bcrypt hash $2…$10$…, not plain text</t>
+          <t>No Admin menu</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>E2E</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
@@ -3187,27 +3167,27 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-20</t>
+          <t>TC-F1-19</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>NFR-01/AC-02</t>
+          <t>NFR-01/AC-01</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Any form</t>
+          <t>New account saved</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Send invalid data bypassing client</t>
+          <t>Inspect users.password_hash in DB</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Server rejects, nothing stored</t>
+          <t>bcrypt hash $2…$10$…, not plain text</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
@@ -3229,32 +3209,32 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-21</t>
+          <t>TC-F1-20</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>NFR-01/AC-03</t>
+          <t>NFR-01/AC-02</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Register form</t>
+          <t>Any form</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Name 101 chars; password 65 chars</t>
+          <t>Send invalid data bypassing client</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>Rejected (100 / 64 accepted)</t>
+          <t>Server rejects, nothing stored</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
@@ -3271,37 +3251,37 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-22</t>
+          <t>TC-F1-21</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>NFR-03/AC-01</t>
+          <t>NFR-01/AC-03</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>develop deployed</t>
+          <t>Register form</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Open public URL</t>
+          <t>Name 101 chars; password 65 chars</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>Home page over HTTPS</t>
+          <t>Rejected (100 / 64 accepted)</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Not run (needs hosting)</t>
+          <t>Pass (30/10)</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
@@ -3313,27 +3293,27 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-23</t>
+          <t>TC-F1-22</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>NFR-03/AC-02</t>
+          <t>NFR-03/AC-01</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Site idle ≥ 15 min</t>
+          <t>develop deployed</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Open URL</t>
+          <t>Open public URL</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Responds; URL recorded</t>
+          <t>Home page over HTTPS</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
@@ -3355,112 +3335,226 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
+          <t>TC-F1-23</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>NFR-03/AC-02</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Site idle ≥ 15 min</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Open URL</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Responds; URL recorded</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>Not run (needs hosting)</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
           <t>TC-F1-24</t>
         </is>
       </c>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>NFR-03/AC-03</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>17/11/2026</t>
         </is>
       </c>
-      <c r="D32" s="5" t="inlineStr">
+      <c r="D33" s="5" t="inlineStr">
         <is>
           <t>Open URL</t>
         </is>
       </c>
-      <c r="E32" s="5" t="inlineStr">
+      <c r="E33" s="5" t="inlineStr">
         <is>
           <t>Online</t>
         </is>
       </c>
-      <c r="F32" s="5" t="inlineStr">
+      <c r="F33" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G32" s="5" t="inlineStr">
+      <c r="G33" s="5" t="inlineStr">
         <is>
           <t>Not run (needs hosting)</t>
         </is>
       </c>
-      <c r="H32" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-    </row>
-    <row r="33"/>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+    </row>
+    <row r="34"/>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Defects found</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Found</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>DEF-F1-01</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>TC-F1-15</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>30/10/2026, manual run (Đạt)</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Any admin URL redirected to /login?next=%2Fadmin: the admin layout guard used a fixed default path, so after login the user landed on the dashboard instead of the page requested. The automated check only tested for next= and missed it</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>src/middleware.js passes the requested path; requireAdmin uses it; E2E now asserts the exact next</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>Fixed, re-verified locally (curl); manual re-test TBD</t>
+        </is>
+      </c>
+    </row>
+    <row r="38"/>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>Summary (local automated)</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>ACs</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>Test cases</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>Executed</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="D40" s="4" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
+      <c r="E40" s="4" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
       </c>
-      <c r="F35" s="4" t="inlineStr">
+      <c r="F40" s="4" t="inlineStr">
         <is>
           <t>Not run</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B41" s="5" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr">
+      <c r="C41" s="5" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="D36" s="5" t="inlineStr">
+      <c r="D41" s="5" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="E36" s="5" t="inlineStr">
+      <c r="E41" s="5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="F36" s="5" t="inlineStr">
+      <c r="F41" s="5" t="inlineStr">
         <is>
           <t>3 (NFR-03 hosting)</t>
         </is>

</xml_diff>

<commit_message>
chore(plan): regenerate Sprint 1 deliverables and update status
Refs: P11
</commit_message>
<xml_diff>
--- a/deliverables/S1/HK261_SPM_FP_Team6_c2_SprintBacklog_S1.xlsx
+++ b/deliverables/S1/HK261_SPM_FP_Team6_c2_SprintBacklog_S1.xlsx
@@ -2264,7 +2264,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -2272,7 +2272,7 @@
     <col width="33" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="53" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
   </cols>
@@ -2336,122 +2336,102 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Hồ Du Tuấn Đạt (AI-assisted)</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Manual run found defect DEF-F1-01 (TC-F1-15); expected result made precise; E2E assertion tightened</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Version history</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>TC</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>AC</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Given</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>When (steps)</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>Then (expected)</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>Automated</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>Actual – local automated</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>Actual – hosted, manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>TC-F1-01</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>US-01/AC-01</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Register page open</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Submit valid name, new email, password Reader2026</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Account created as Customer, signed in, redirected home</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>E2E + INT</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>Pass (30/10)</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-02</t>
+          <t>TC-F1-01</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>US-01/AC-02</t>
+          <t>US-01/AC-01</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Customer x@y.com exists</t>
+          <t>Register page open</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Register with X@Y.COM</t>
+          <t>Submit valid name, new email, password Reader2026</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>"Email is already registered" by email field; no new account</t>
+          <t>Account created as Customer, signed in, redirected home</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -2473,27 +2453,27 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-03</t>
+          <t>TC-F1-02</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>US-01/AC-03</t>
+          <t>US-01/AC-02</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Register page open</t>
+          <t>Customer x@y.com exists</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Submit not-an-email; then empty fields; then POST bypassing client</t>
+          <t>Register with X@Y.COM</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Field errors on client; server also rejects</t>
+          <t>"Email is already registered" by email field; no new account</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -2515,12 +2495,12 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-04</t>
+          <t>TC-F1-03</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>US-01/AC-04</t>
+          <t>US-01/AC-03</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -2530,17 +2510,17 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Password abc1234 (7) then abcd1234 (8)</t>
+          <t>Submit not-an-email; then empty fields; then POST bypassing client</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>7 rejected, 8 accepted</t>
+          <t>Field errors on client; server also rejects</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>E2E + UNIT</t>
+          <t>E2E + INT</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -2557,32 +2537,32 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-05</t>
+          <t>TC-F1-04</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>US-02/AC-01</t>
+          <t>US-01/AC-04</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Active account</t>
+          <t>Register page open</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Log in with correct credentials</t>
+          <t>Password abc1234 (7) then abcd1234 (8)</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Signed in; name and Log out shown</t>
+          <t>7 rejected, 8 accepted</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>E2E + INT</t>
+          <t>E2E + UNIT</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -2599,12 +2579,12 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-06</t>
+          <t>TC-F1-05</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>US-02/AC-02</t>
+          <t>US-02/AC-01</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -2614,12 +2594,12 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Log in with wrong password; with unknown email</t>
+          <t>Log in with correct credentials</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Same generic "Invalid email or password"</t>
+          <t>Signed in; name and Log out shown</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -2641,27 +2621,27 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-07</t>
+          <t>TC-F1-06</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>US-02/AC-03</t>
+          <t>US-02/AC-02</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Account locked by admin</t>
+          <t>Active account</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Log in with correct credentials</t>
+          <t>Log in with wrong password; with unknown email</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>"This account is locked…"</t>
+          <t>Same generic "Invalid email or password"</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
@@ -2683,32 +2663,32 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-08</t>
+          <t>TC-F1-07</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>US-02/AC-04</t>
+          <t>US-02/AC-03</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Signed in</t>
+          <t>Account locked by admin</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Click Log out; open /admin</t>
+          <t>Log in with correct credentials</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Session ended; redirected to Login</t>
+          <t>"This account is locked…"</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>E2E</t>
+          <t>E2E + INT</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -2725,32 +2705,32 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-09</t>
+          <t>TC-F1-08</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>US-02/AC-05</t>
+          <t>US-02/AC-04</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Account e@x.com</t>
+          <t>Signed in</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Log in with   E@X.COM </t>
+          <t>Click Log out; open /admin</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Signed in</t>
+          <t>Session ended; redirected to Login</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>E2E + INT + UNIT</t>
+          <t>E2E</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -2767,32 +2747,32 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-10</t>
+          <t>TC-F1-09</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>US-03/AC-01</t>
+          <t>US-02/AC-05</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Signed in as admin</t>
+          <t>Account e@x.com</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Create account with role Customer</t>
+          <t xml:space="preserve">Log in with   E@X.COM </t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Appears in list, role Customer, Active</t>
+          <t>Signed in</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>E2E + INT</t>
+          <t>E2E + INT + UNIT</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -2809,27 +2789,27 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-11</t>
+          <t>TC-F1-10</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>US-03/AC-02</t>
+          <t>US-03/AC-01</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Admin; another active account</t>
+          <t>Signed in as admin</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Lock, then Unlock</t>
+          <t>Create account with role Customer</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Locked user cannot log in; after unlock can</t>
+          <t>Appears in list, role Customer, Active</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
@@ -2851,27 +2831,27 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-12</t>
+          <t>TC-F1-11</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>US-03/AC-03</t>
+          <t>US-03/AC-02</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Signed in as admin</t>
+          <t>Admin; another active account</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Click Lock on own row</t>
+          <t>Lock, then Unlock</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>"You cannot lock your own account"</t>
+          <t>Locked user cannot log in; after unlock can</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
@@ -2893,27 +2873,27 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-13</t>
+          <t>TC-F1-12</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>US-03/AC-04</t>
+          <t>US-03/AC-03</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Admin; email exists</t>
+          <t>Signed in as admin</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Create account with that email</t>
+          <t>Click Lock on own row</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Field error; no account</t>
+          <t>"You cannot lock your own account"</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
@@ -2935,27 +2915,27 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-14</t>
+          <t>TC-F1-13</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>US-03/AC-05</t>
+          <t>US-03/AC-04</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>User signed in in another browser</t>
+          <t>Admin; email exists</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Admin locks that user; user reloads</t>
+          <t>Create account with that email</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>User is signed out</t>
+          <t>Field error; no account</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
@@ -2977,32 +2957,32 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-15</t>
+          <t>TC-F1-14</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>US-04/AC-01</t>
+          <t>US-03/AC-05</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Not signed in</t>
+          <t>User signed in in another browser</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Open /admin/accounts</t>
+          <t>Admin locks that user; user reloads</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Redirect to /login?next=…</t>
+          <t>User is signed out</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>E2E</t>
+          <t>E2E + INT</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
@@ -3019,27 +2999,27 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-16</t>
+          <t>TC-F1-15</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>US-04/AC-02</t>
+          <t>US-04/AC-01</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Signed in as Customer</t>
+          <t>Not signed in</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Open /admin/accounts directly</t>
+          <t>Open /admin/accounts</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>HTTP 403 "Access denied"</t>
+          <t>Redirect to /login?next=%2Fadmin%2Faccounts; after login back on that page</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
@@ -3061,27 +3041,27 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-17</t>
+          <t>TC-F1-16</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>US-04/AC-03</t>
+          <t>US-04/AC-02</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Signed in as admin</t>
+          <t>Signed in as Customer</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Open /admin</t>
+          <t>Open /admin/accounts directly</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Admin dashboard shown</t>
+          <t>HTTP 403 "Access denied"</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
@@ -3103,27 +3083,27 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-18</t>
+          <t>TC-F1-17</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>US-04/AC-04</t>
+          <t>US-04/AC-03</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Signed in as Customer</t>
+          <t>Signed in as admin</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Look at header on any page</t>
+          <t>Open /admin</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>No Admin menu</t>
+          <t>Admin dashboard shown</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
@@ -3145,32 +3125,32 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-19</t>
+          <t>TC-F1-18</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>NFR-01/AC-01</t>
+          <t>US-04/AC-04</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>New account saved</t>
+          <t>Signed in as Customer</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Inspect users.password_hash in DB</t>
+          <t>Look at header on any page</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>bcrypt hash $2…$10$…, not plain text</t>
+          <t>No Admin menu</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>E2E</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
@@ -3187,27 +3167,27 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-20</t>
+          <t>TC-F1-19</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>NFR-01/AC-02</t>
+          <t>NFR-01/AC-01</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Any form</t>
+          <t>New account saved</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Send invalid data bypassing client</t>
+          <t>Inspect users.password_hash in DB</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Server rejects, nothing stored</t>
+          <t>bcrypt hash $2…$10$…, not plain text</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
@@ -3229,32 +3209,32 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-21</t>
+          <t>TC-F1-20</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>NFR-01/AC-03</t>
+          <t>NFR-01/AC-02</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Register form</t>
+          <t>Any form</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Name 101 chars; password 65 chars</t>
+          <t>Send invalid data bypassing client</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>Rejected (100 / 64 accepted)</t>
+          <t>Server rejects, nothing stored</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
@@ -3271,37 +3251,37 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-22</t>
+          <t>TC-F1-21</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>NFR-03/AC-01</t>
+          <t>NFR-01/AC-03</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>develop deployed</t>
+          <t>Register form</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Open public URL</t>
+          <t>Name 101 chars; password 65 chars</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>Home page over HTTPS</t>
+          <t>Rejected (100 / 64 accepted)</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>UNIT</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Not run (needs hosting)</t>
+          <t>Pass (30/10)</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
@@ -3313,27 +3293,27 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>TC-F1-23</t>
+          <t>TC-F1-22</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>NFR-03/AC-02</t>
+          <t>NFR-03/AC-01</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Site idle ≥ 15 min</t>
+          <t>develop deployed</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Open URL</t>
+          <t>Open public URL</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Responds; URL recorded</t>
+          <t>Home page over HTTPS</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
@@ -3355,112 +3335,226 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
+          <t>TC-F1-23</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>NFR-03/AC-02</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Site idle ≥ 15 min</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Open URL</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Responds; URL recorded</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>Not run (needs hosting)</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
           <t>TC-F1-24</t>
         </is>
       </c>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>NFR-03/AC-03</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>17/11/2026</t>
         </is>
       </c>
-      <c r="D32" s="5" t="inlineStr">
+      <c r="D33" s="5" t="inlineStr">
         <is>
           <t>Open URL</t>
         </is>
       </c>
-      <c r="E32" s="5" t="inlineStr">
+      <c r="E33" s="5" t="inlineStr">
         <is>
           <t>Online</t>
         </is>
       </c>
-      <c r="F32" s="5" t="inlineStr">
+      <c r="F33" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G32" s="5" t="inlineStr">
+      <c r="G33" s="5" t="inlineStr">
         <is>
           <t>Not run (needs hosting)</t>
         </is>
       </c>
-      <c r="H32" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-    </row>
-    <row r="33"/>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+    </row>
+    <row r="34"/>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Defects found</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Found</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>DEF-F1-01</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>TC-F1-15</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>30/10/2026, manual run (Đạt)</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Any admin URL redirected to /login?next=%2Fadmin: the admin layout guard used a fixed default path, so after login the user landed on the dashboard instead of the page requested. The automated check only tested for next= and missed it</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>src/middleware.js passes the requested path; requireAdmin uses it; E2E now asserts the exact next</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>Fixed, re-verified locally (curl); manual re-test TBD</t>
+        </is>
+      </c>
+    </row>
+    <row r="38"/>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>Summary (local automated)</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>ACs</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>Test cases</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>Executed</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="D40" s="4" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
+      <c r="E40" s="4" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
       </c>
-      <c r="F35" s="4" t="inlineStr">
+      <c r="F40" s="4" t="inlineStr">
         <is>
           <t>Not run</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B41" s="5" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr">
+      <c r="C41" s="5" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="D36" s="5" t="inlineStr">
+      <c r="D41" s="5" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="E36" s="5" t="inlineStr">
+      <c r="E41" s="5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="F36" s="5" t="inlineStr">
+      <c r="F41" s="5" t="inlineStr">
         <is>
           <t>3 (NFR-03 hosting)</t>
         </is>
@@ -4456,14 +4550,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F90"/>
+  <dimension ref="A1:F92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="49" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="37" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -4555,158 +4649,153 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>1.1-draft</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Nguyễn Minh Chính (PO, AI-assisted)</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Roles confirmed; capacity 20 h per member per Sprint adopted as plan value (40 h/Sprint, 120 h, BAC 24.0 M VND); CR-06 Option B recommended; Excel version added</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>3.2 Milestones (fixed by the brief)</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Milestone</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Date / time (GMT+7)</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Evidence</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>Source</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>M0</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Project start, brief issued</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Fri 23/10</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>[03 §5]</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>M0</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>CR-06 issued by Sponsor</t>
+          <t>Project start, brief issued</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Tue 27/10</t>
+          <t>Fri 23/10</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>CR-06 in Change Log</t>
+          <t>–</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>[CR-06]</t>
+          <t>[03 §5]</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Sprint 1 submission (c1, c2, c3, c0)</t>
+          <t>CR-06 issued by Sponsor</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Thu 29/10 23:59</t>
+          <t>Tue 27/10</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>eLearning upload</t>
+          <t>CR-06 in Change Log</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>[03 §7]</t>
+          <t>[CR-06]</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Review/Retro 1 + CCB for CR-06</t>
+          <t>Sprint 1 submission (c1, c2, c3, c0)</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Fri 30/10</t>
+          <t>Thu 29/10 23:59</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Review slides, CCB decision</t>
+          <t>eLearning upload</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>[03 §5], [CR-06 §5]</t>
+          <t>[03 §7]</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Baseline v1.0 tagged (baseline-v1.0)</t>
+          <t>Review/Retro 1 + CCB for CR-06</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -4716,423 +4805,433 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Git tag</t>
+          <t>Review slides, CCB decision</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>PMP-6</t>
+          <t>[03 §5], [CR-06 §5]</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Sprint 2 submission (c2, c3, c4 CR, c0)</t>
+          <t>Baseline v1.0 tagged (baseline-v1.0)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Thu 05/11 23:59</t>
+          <t>Fri 30/10</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>eLearning upload</t>
+          <t>Git tag</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>[03 §7]</t>
+          <t>PMP-6</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>M6</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Review/Retro 2</t>
+          <t>Sprint 2 submission (c2, c3, c4 CR, c0)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Fri 06/11</t>
+          <t>Thu 05/11 23:59</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Review slides</t>
+          <t>eLearning upload</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>[03 §5]</t>
+          <t>[03 §7]</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>M7</t>
+          <t>M6</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Release v1.0 tagged + release notes</t>
+          <t>Review/Retro 2</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Thu 12/11</t>
+          <t>Fri 06/11</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Git tag, notes</t>
+          <t>Review slides</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>[03 §6.3]</t>
+          <t>[03 §5]</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>M7</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Sprint 3 submission (c2, c3, c5 UAT, c0)</t>
+          <t>Release v1.0 tagged + release notes</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Thu 12/11 23:59</t>
+          <t>Thu 12/11</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>eLearning upload</t>
+          <t>Git tag, notes</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>[03 §7]</t>
+          <t>[03 §6.3]</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>M9</t>
+          <t>M8</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Review 3 + UAT with customer</t>
+          <t>Sprint 3 submission (c2, c3, c5 UAT, c0)</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Fri 13/11</t>
+          <t>Thu 12/11 23:59</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Signed UAT minutes</t>
+          <t>eLearning upload</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>[03 §6.3]</t>
+          <t>[03 §7]</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>M10</t>
+          <t>M9</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Final submission (c1 Final, c2 Final, c6 Report, c6 Slides, Eval360)</t>
+          <t>Review 3 + UAT with customer</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Sun 15/11 23:59</t>
+          <t>Fri 13/11</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>eLearning upload</t>
+          <t>Signed UAT minutes</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>[03 §7]</t>
+          <t>[03 §6.3]</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Final submission (c1 Final, c2 Final, c6 Report, c6 Slides, Eval360)</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Sun 15/11 23:59</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>eLearning upload</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>[03 §7]</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
           <t>M11</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>Final presentation; site online until end of day</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>Tue 17/11 07:00</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>Live demo</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>[03 §8]</t>
         </is>
       </c>
     </row>
-    <row r="23"/>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+    <row r="24"/>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>3.3 Sprint plan and leader rotation</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Sprint</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>Dates</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>Leader</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>Sprint Goal (plan)</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>Increment</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>PM focus (rubric S4)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>S1 – Plan baseline &amp; F1</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>23/10 – 29/10</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Hồ Du Tuấn Đạt *(to confirm)*</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>"Users can register, log in and log out; an administrator can create and lock accounts; non-admins are blocked from admin functions on the server."</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>PMP v1.0</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>S2 – Execution, monitoring &amp; change</t>
+          <t>S1 – Plan baseline &amp; F1</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>30/10 – 05/11</t>
+          <t>23/10 – 29/10</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Nguyễn Minh Chính (PO) *(to confirm)*</t>
+          <t>Hồ Du Tuấn Đạt</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>"Admins manage books, categories and authors (soft delete), and customers browse 12 books per page, newest first, on any device." (+ CR-06 if approved)</t>
+          <t>"Users can register, log in and log out; an administrator can create and lock accounts; non-admins are blocked from admin functions on the server."</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>F2, F3 (+CR-06)</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>CR + risk/issue</t>
+          <t>PMP v1.0</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>S3 – Complete &amp; acceptance</t>
+          <t>S2 – Execution, monitoring &amp; change</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>06/11 – 12/11</t>
+          <t>30/10 – 05/11</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Hồ Du Tuấn Đạt *(to confirm)*</t>
+          <t>Nguyễn Minh Chính (PO)</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>"Customers open book details and search/filter by title, author, category and price range together with pagination; Release v1.0 passes UAT."</t>
+          <t>"Admins manage books, categories and authors (soft delete), and customers browse 12 books per page, newest first, on any device." (+ CR-06 if approved)</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>F4, F5</t>
+          <t>F2, F3 (+CR-06)</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>UAT + Release</t>
+          <t>CR + risk/issue</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
+          <t>S3 – Complete &amp; acceptance</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>06/11 – 12/11</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Hồ Du Tuấn Đạt</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>"Customers open book details and search/filter by title, author, category and price range together with pagination; Release v1.0 passes UAT."</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>F4, F5</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>UAT + Release</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
           <t>Closure</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>13/11 – 17/11</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>Final Report, EVM, Lessons Learned, slides, video</t>
         </is>
       </c>
-      <c r="E29" s="5" t="inlineStr">
+      <c r="E30" s="5" t="inlineStr">
         <is>
           <t>Release 1.0 online</t>
         </is>
       </c>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="F30" s="5" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
     </row>
-    <row r="30"/>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+    <row r="31"/>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>3.4 Allocation of backlog items to Sprints (plan)</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>Sprint</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>Items</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>SP (plan)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>US-01 Register · US-02 Log in/out · US-03 Admin creates &amp; locks accounts · US-04 Server-side role guard · NFR-01 Password hashing &amp; validation · NFR-03 Hosting/deploy skeleton</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>US-05 Add book · US-06 Edit book · US-07 Hide (soft delete) book · US-08 Manage categories · US-09 Manage authors · NFR-02 Seed ≥30 books · US-10 Book grid 12/page newest first · NFR-04 Responsive UI</t>
+          <t>US-01 Register · US-02 Log in/out · US-03 Admin creates &amp; locks accounts · US-04 Server-side role guard · NFR-01 Password hashing &amp; validation · NFR-03 Hosting/deploy skeleton</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
@@ -5144,12 +5243,12 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>S2 (if CR-06 approved, option per CCB)</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>US-24 Store Staff role &amp; permissions · US-25 "Last updated by" audit</t>
+          <t>US-05 Add book · US-06 Edit book · US-07 Hide (soft delete) book · US-08 Manage categories · US-09 Manage authors · NFR-02 Seed ≥30 books · US-10 Book grid 12/page newest first · NFR-04 Responsive UI</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
@@ -5161,12 +5260,12 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>S3</t>
+          <t>S2 (if CR-06 approved, option per CCB)</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>US-11 Book detail page (+friendly not-found, Back keeps page) · US-12 Search by title/author · US-13 Filter by category &amp; price range with pagination · NFR-05 List page &lt; 2 s</t>
+          <t>US-24 Store Staff role &amp; permissions · US-25 "Last updated by" audit</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
@@ -5178,244 +5277,220 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>US-11 Book detail page (+friendly not-found, Back keeps page) · US-12 Search by title/author · US-13 Filter by category &amp; price range with pagination · NFR-05 List page &lt; 2 s</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
           <t>Release 1.0 total</t>
         </is>
       </c>
-      <c r="B37" s="5" t="inlineStr"/>
-      <c r="C37" s="5" t="inlineStr">
+      <c r="B38" s="5" t="inlineStr"/>
+      <c r="C38" s="5" t="inlineStr">
         <is>
           <t>PSP = TBD</t>
         </is>
       </c>
     </row>
-    <row r="38"/>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
+    <row r="39"/>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
         <is>
           <t>3.5 Capacity and expected velocity</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t>Sprint</t>
         </is>
       </c>
-      <c r="B40" s="4" t="inlineStr">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>Đạt (h)</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr">
+      <c r="C41" s="4" t="inlineStr">
         <is>
           <t>Chính (h)</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="D41" s="4" t="inlineStr">
         <is>
           <t>Capacity (h)</t>
         </is>
       </c>
-      <c r="E40" s="4" t="inlineStr">
+      <c r="E41" s="4" t="inlineStr">
         <is>
           <t>Source</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>plan/INPUTS.md §2</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr"/>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>plan/INPUTS.md §2 (plan value, PO 30/10/2026)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
           <t>S3</t>
         </is>
       </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr"/>
-    </row>
-    <row r="44"/>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr"/>
+    </row>
     <row r="45">
-      <c r="A45" s="3" t="inlineStr">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr"/>
+    </row>
+    <row r="46"/>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>3.7 Master schedule (work packages by date)</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="B46" s="4" t="inlineStr">
+      <c r="B48" s="4" t="inlineStr">
         <is>
           <t>Work package</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C48" s="4" t="inlineStr">
         <is>
           <t>Start</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="D48" s="4" t="inlineStr">
         <is>
           <t>Due</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="E48" s="4" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="F46" s="4" t="inlineStr">
+      <c r="F48" s="4" t="inlineStr">
         <is>
           <t>Depends on</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
-        <is>
-          <t>Sprint 1 (23–29/10)</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
-        <is>
-          <t>P00</t>
-        </is>
-      </c>
-      <c r="B48" s="5" t="inlineStr">
-        <is>
-          <t>Repo, branches, access (GV invited)</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>27/10</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>27/10</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>Đạt</t>
-        </is>
-      </c>
-      <c r="F48" s="5" t="inlineStr">
-        <is>
-          <t>–</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>P01</t>
-        </is>
-      </c>
-      <c r="B49" s="5" t="inlineStr">
-        <is>
-          <t>Kick-off, roles, working agreement, capacity</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>27/10</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>28/10</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F49" s="5" t="inlineStr">
-        <is>
-          <t>P00</t>
+          <t>Sprint 1 (23–29/10)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>P00</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>Product Backlog v1.0 (GWT, DoR)</t>
+          <t>Repo, branches, access (GV invited)</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
@@ -5425,61 +5500,61 @@
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>28/10</t>
+          <t>27/10</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>PO</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>P01</t>
+          <t>–</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>P03</t>
+          <t>P01</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Planning Poker, Release Plan, BAC</t>
+          <t>Kick-off, roles, working agreement, capacity</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
+          <t>27/10</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
           <t>28/10</t>
         </is>
       </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>28/10</t>
-        </is>
-      </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>PO + Leader</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>P00</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>P02</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Stack, scaffold, deploy skeleton</t>
+          <t>Product Backlog v1.0 (GWT, DoR)</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
@@ -5494,7 +5569,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>Đạt</t>
+          <t>PO</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
@@ -5506,12 +5581,12 @@
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>P03</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>Sprint Planning 1 → Jira</t>
+          <t>Planning Poker, Release Plan, BAC</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
@@ -5526,88 +5601,88 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>Leader</t>
+          <t>PO + Leader</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>P03</t>
+          <t>P02</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>P06–P07</t>
+          <t>P04</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>Build F1; F1 test cases</t>
+          <t>Stack, scaffold, deploy skeleton</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
+          <t>27/10</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
           <t>28/10</t>
         </is>
       </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>29/10</t>
-        </is>
-      </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>P04, P05</t>
+          <t>P01</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>PMP v1.0 (7 parts)</t>
+          <t>Sprint Planning 1 → Jira</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>27/10</t>
+          <t>28/10</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>29/10</t>
+          <t>28/10</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>Leader + PO</t>
+          <t>Leader</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>P01, P03</t>
+          <t>P03</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P06–P07</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>CR-06 Change Log, impact analysis, options</t>
+          <t>Build F1; F1 test cases</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
@@ -5622,29 +5697,29 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t>PO</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>P03</t>
+          <t>P04, P05</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>Daily log, burndown, actual hours</t>
+          <t>PMP v1.0 (7 parts)</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>23/10</t>
+          <t>27/10</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
@@ -5654,95 +5729,120 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t>Leader</t>
+          <t>Leader + PO</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>continuous</t>
+          <t>P01, P03</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P09</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>Package &amp; submit S1</t>
+          <t>CR-06 Change Log, impact analysis, options</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
+          <t>28/10</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
           <t>29/10</t>
         </is>
       </c>
-      <c r="D58" s="5" t="inlineStr">
-        <is>
-          <t>29/10 23:59</t>
-        </is>
-      </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t>Leader</t>
+          <t>PO</t>
         </is>
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>above</t>
+          <t>P03</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>Review/Retro 1 + CCB</t>
+          <t>Daily log, burndown, actual hours</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>30/10</t>
+          <t>23/10</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>30/10</t>
+          <t>29/10</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t>Leader + PO</t>
+          <t>Leader</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>continuous</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>Sprint 2 (30/10–05/11)</t>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>Package &amp; submit S1</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>29/10</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>29/10 23:59</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>Leader</t>
+        </is>
+      </c>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>above</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>P12</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>Sprint Planning 2 (actual velocity S1)</t>
+          <t>Review/Retro 1 + CCB</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
@@ -5757,130 +5857,105 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>Leader</t>
+          <t>Leader + PO</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>P11</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>P14</t>
-        </is>
-      </c>
-      <c r="B62" s="5" t="inlineStr">
-        <is>
-          <t>Update baseline per CCB, tag</t>
-        </is>
-      </c>
-      <c r="C62" s="5" t="inlineStr">
-        <is>
-          <t>30/10</t>
-        </is>
-      </c>
-      <c r="D62" s="5" t="inlineStr">
-        <is>
-          <t>31/10</t>
-        </is>
-      </c>
-      <c r="E62" s="5" t="inlineStr">
-        <is>
-          <t>PO</t>
-        </is>
-      </c>
-      <c r="F62" s="5" t="inlineStr">
-        <is>
-          <t>CCB decision</t>
+          <t>Sprint 2 (30/10–05/11)</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>P15</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>Build F2 (+ seed ≥30 books)</t>
+          <t>Sprint Planning 2 (actual velocity S1)</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>31/10</t>
+          <t>30/10</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>03/11</t>
+          <t>30/10</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Leader</t>
         </is>
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>P12</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>Build F3</t>
+          <t>Update baseline per CCB, tag</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>02/11</t>
+          <t>30/10</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>04/11</t>
+          <t>31/10</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>PO</t>
         </is>
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>P15</t>
+          <t>CCB decision</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>P17</t>
+          <t>P15</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>Build CR-06 (if approved)</t>
+          <t>Build F2 (+ seed ≥30 books)</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>01/11</t>
+          <t>31/10</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>04/11</t>
+          <t>03/11</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -5890,29 +5965,29 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>P13</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>P18</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>Test cases F2, F3, CR-06 + regression F1</t>
+          <t>Build F3</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>03/11</t>
+          <t>02/11</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>05/11</t>
+          <t>04/11</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -5922,56 +5997,56 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>P15–P17</t>
+          <t>P15</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>P19</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>Weekly Status, risk &amp; issue log</t>
+          <t>Build CR-06 (if approved)</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>30/10</t>
+          <t>01/11</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>05/11</t>
+          <t>04/11</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t>Leader</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>continuous</t>
+          <t>P14</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>P20</t>
+          <t>P18</t>
         </is>
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>c4 Change Request form</t>
+          <t>Test cases F2, F3, CR-06 + regression F1</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>31/10</t>
+          <t>03/11</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
@@ -5981,36 +6056,36 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t>PO</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>P15–P17</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>P21</t>
+          <t>P19</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>Package &amp; submit S2</t>
+          <t>Weekly Status, risk &amp; issue log</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
+          <t>30/10</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
           <t>05/11</t>
         </is>
       </c>
-      <c r="D69" s="5" t="inlineStr">
-        <is>
-          <t>05/11 23:59</t>
-        </is>
-      </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
           <t>Leader</t>
@@ -6018,58 +6093,83 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>above</t>
+          <t>continuous</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>P22</t>
+          <t>P20</t>
         </is>
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>Review/Retro 2</t>
+          <t>c4 Change Request form</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>06/11</t>
+          <t>31/10</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>06/11</t>
+          <t>05/11</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t>Leader</t>
+          <t>PO</t>
         </is>
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>P21</t>
+          <t>P14</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>Sprint 3 (06–12/11)</t>
+          <t>P21</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>Package &amp; submit S2</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>05/11</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>05/11 23:59</t>
+        </is>
+      </c>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>Leader</t>
+        </is>
+      </c>
+      <c r="F71" s="5" t="inlineStr">
+        <is>
+          <t>above</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>P23</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>Sprint Planning 3 (actual velocity S2)</t>
+          <t>Review/Retro 2</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
@@ -6089,115 +6189,90 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>P22</t>
+          <t>P21</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>P24–P25</t>
-        </is>
-      </c>
-      <c r="B73" s="5" t="inlineStr">
-        <is>
-          <t>Build F4, F5</t>
-        </is>
-      </c>
-      <c r="C73" s="5" t="inlineStr">
-        <is>
-          <t>07/11</t>
-        </is>
-      </c>
-      <c r="D73" s="5" t="inlineStr">
-        <is>
-          <t>10/11</t>
-        </is>
-      </c>
-      <c r="E73" s="5" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F73" s="5" t="inlineStr">
-        <is>
-          <t>P23</t>
+          <t>Sprint 3 (06–12/11)</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>P26</t>
+          <t>P23</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>Tests F4, F5, regression F1–F3, performance</t>
+          <t>Sprint Planning 3 (actual velocity S2)</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>10/11</t>
+          <t>06/11</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>11/11</t>
+          <t>06/11</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Leader</t>
         </is>
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>P24, P25</t>
+          <t>P22</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>P27</t>
+          <t>P24–P25</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>Release v1.0: merge to main, tag, notes</t>
+          <t>Build F4, F5</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>11/11</t>
+          <t>07/11</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>12/11</t>
+          <t>10/11</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t>Leader</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>P26</t>
+          <t>P23</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>P28</t>
+          <t>P26</t>
         </is>
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>UAT script (all ACs)</t>
+          <t>Tests F4, F5, regression F1–F3, performance</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
@@ -6207,34 +6282,34 @@
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>12/11</t>
+          <t>11/11</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t>PO</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>P26</t>
+          <t>P24, P25</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>P29</t>
+          <t>P27</t>
         </is>
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>Monitoring + draft EVM</t>
+          <t>Release v1.0: merge to main, tag, notes</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>06/11</t>
+          <t>11/11</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
@@ -6249,90 +6324,115 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>continuous</t>
+          <t>P26</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>P30</t>
+          <t>P28</t>
         </is>
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>Package &amp; submit S3</t>
+          <t>UAT script (all ACs)</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
+          <t>10/11</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
           <t>12/11</t>
         </is>
       </c>
-      <c r="D78" s="5" t="inlineStr">
-        <is>
-          <t>12/11 23:59</t>
-        </is>
-      </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t>Leader</t>
+          <t>PO</t>
         </is>
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>above</t>
+          <t>P26</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>P31</t>
+          <t>P29</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>Review 3 + UAT + minutes</t>
+          <t>Monitoring + draft EVM</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>13/11</t>
+          <t>06/11</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>13/11</t>
+          <t>12/11</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Leader + PO</t>
+          <t>Leader</t>
         </is>
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>P30</t>
+          <t>continuous</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>Closure (13–17/11)</t>
+          <t>P30</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>Package &amp; submit S3</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>12/11</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>12/11 23:59</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>Leader</t>
+        </is>
+      </c>
+      <c r="F80" s="5" t="inlineStr">
+        <is>
+          <t>above</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>P32</t>
+          <t>P31</t>
         </is>
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>Final hosting, demo accounts, closure data</t>
+          <t>Review 3 + UAT + minutes</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
@@ -6342,105 +6442,80 @@
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>14/11</t>
+          <t>13/11</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t>Đạt</t>
+          <t>Leader + PO</t>
         </is>
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>P31</t>
+          <t>P30</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>P33</t>
-        </is>
-      </c>
-      <c r="B82" s="5" t="inlineStr">
-        <is>
-          <t>Final Report, EVM, Lessons Learned, PMP/Workbook Final</t>
-        </is>
-      </c>
-      <c r="C82" s="5" t="inlineStr">
-        <is>
-          <t>13/11</t>
-        </is>
-      </c>
-      <c r="D82" s="5" t="inlineStr">
-        <is>
-          <t>15/11</t>
-        </is>
-      </c>
-      <c r="E82" s="5" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="F82" s="5" t="inlineStr">
-        <is>
-          <t>P31, P32</t>
+          <t>Closure (13–17/11)</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>P34</t>
+          <t>P32</t>
         </is>
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>Slides + demo video ≤ 3 min</t>
+          <t>Final hosting, demo accounts, closure data</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
+          <t>13/11</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
           <t>14/11</t>
         </is>
       </c>
-      <c r="D83" s="5" t="inlineStr">
-        <is>
-          <t>15/11</t>
-        </is>
-      </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>P33</t>
+          <t>P31</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>P35</t>
+          <t>P33</t>
         </is>
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>Final submission + Eval360 each</t>
+          <t>Final Report, EVM, Lessons Learned, PMP/Workbook Final</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
+          <t>13/11</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
           <t>15/11</t>
         </is>
       </c>
-      <c r="D84" s="5" t="inlineStr">
-        <is>
-          <t>15/11 23:59</t>
-        </is>
-      </c>
       <c r="E84" s="5" t="inlineStr">
         <is>
           <t>Both</t>
@@ -6448,141 +6523,205 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>P33, P34</t>
+          <t>P31, P32</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
+          <t>P34</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>Slides + demo video ≤ 3 min</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>14/11</t>
+        </is>
+      </c>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t>15/11</t>
+        </is>
+      </c>
+      <c r="E85" s="5" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F85" s="5" t="inlineStr">
+        <is>
+          <t>P33</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="5" t="inlineStr">
+        <is>
+          <t>P35</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>Final submission + Eval360 each</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>15/11</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>15/11 23:59</t>
+        </is>
+      </c>
+      <c r="E86" s="5" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F86" s="5" t="inlineStr">
+        <is>
+          <t>P33, P34</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="5" t="inlineStr">
+        <is>
           <t>P36</t>
         </is>
       </c>
-      <c r="B85" s="5" t="inlineStr">
+      <c r="B87" s="5" t="inlineStr">
         <is>
           <t>Final presentation</t>
         </is>
       </c>
-      <c r="C85" s="5" t="inlineStr">
+      <c r="C87" s="5" t="inlineStr">
         <is>
           <t>16/11</t>
         </is>
       </c>
-      <c r="D85" s="5" t="inlineStr">
+      <c r="D87" s="5" t="inlineStr">
         <is>
           <t>17/11 07:00</t>
         </is>
       </c>
-      <c r="E85" s="5" t="inlineStr">
+      <c r="E87" s="5" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="F85" s="5" t="inlineStr">
+      <c r="F87" s="5" t="inlineStr">
         <is>
           <t>P35</t>
         </is>
       </c>
     </row>
-    <row r="86"/>
-    <row r="87">
-      <c r="A87" s="3" t="inlineStr">
+    <row r="88"/>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
         <is>
           <t>3.8 Baseline and change history of this plan</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="4" t="inlineStr">
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr">
         <is>
           <t>Baseline</t>
         </is>
       </c>
-      <c r="B88" s="4" t="inlineStr">
+      <c r="B90" s="4" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C88" s="4" t="inlineStr">
+      <c r="C90" s="4" t="inlineStr">
         <is>
           <t>Trigger</t>
         </is>
       </c>
-      <c r="D88" s="4" t="inlineStr">
+      <c r="D90" s="4" t="inlineStr">
         <is>
           <t>PSP</t>
         </is>
       </c>
-      <c r="E88" s="4" t="inlineStr">
+      <c r="E90" s="4" t="inlineStr">
         <is>
           <t>BAC</t>
         </is>
       </c>
-      <c r="F88" s="4" t="inlineStr">
+      <c r="F90" s="4" t="inlineStr">
         <is>
           <t>Tag</t>
         </is>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" s="5" t="inlineStr">
+    <row r="91">
+      <c r="A91" s="5" t="inlineStr">
         <is>
           <t>Baseline v1.0</t>
         </is>
       </c>
-      <c r="B89" s="5" t="inlineStr">
+      <c r="B91" s="5" t="inlineStr">
         <is>
           <t>30/10/2026</t>
         </is>
       </c>
-      <c r="C89" s="5" t="inlineStr">
+      <c r="C91" s="5" t="inlineStr">
         <is>
           <t>Sprint 1 submission</t>
         </is>
       </c>
-      <c r="D89" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E89" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F89" s="5" t="inlineStr">
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E91" s="5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F91" s="5" t="inlineStr">
         <is>
           <t>baseline-v1.0</t>
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="5" t="inlineStr">
+    <row r="92">
+      <c r="A92" s="5" t="inlineStr">
         <is>
           <t>Rebaseline v1.1</t>
         </is>
       </c>
-      <c r="B90" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C90" s="5" t="inlineStr">
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
         <is>
           <t>CCB decision on CR-06 (if Approve)</t>
         </is>
       </c>
-      <c r="D90" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E90" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F90" s="5" t="inlineStr">
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E92" s="5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F92" s="5" t="inlineStr">
         <is>
           <t>baseline-v1.1</t>
         </is>
@@ -6737,17 +6876,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>20 (plan)</t>
         </is>
       </c>
     </row>
@@ -6759,17 +6898,17 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>20 (plan)</t>
         </is>
       </c>
     </row>
@@ -6783,7 +6922,7 @@
       <c r="C13" s="5" t="inlineStr"/>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>TBD (scenario 40 h, PMP-3 §3.5)</t>
+          <t>40 (plan) – plan/INPUTS.md §2, PO 30/10/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(backlog): record PO story-point estimates, PSP 55 and expected velocity
Estimates set by the PO from AI-suggested values; no voting rounds held (planning-poker-log v1.1). Refs: P03
</commit_message>
<xml_diff>
--- a/deliverables/S1/HK261_SPM_FP_Team6_c2_SprintBacklog_S1.xlsx
+++ b/deliverables/S1/HK261_SPM_FP_Team6_c2_SprintBacklog_S1.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>TBD after Planning Poker</t>
+          <t>55 (S1 18 · S2 24 · S3 13)</t>
         </is>
       </c>
     </row>
@@ -535,7 +535,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -569,7 +569,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>PSP = TBD</t>
+          <t>PSP = 55 (baseline v1.0; 62 if CR-06 is approved)</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -777,7 +777,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -819,7 +819,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
@@ -945,7 +945,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -987,7 +987,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
@@ -1029,7 +1029,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -3794,14 +3794,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -3871,671 +3871,777 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Session 1 – Release 1.0 baseline (date: TBD, place/tool: TBD, facilitator: PO)</t>
-        </is>
-      </c>
-    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Nguyễn Minh Chính (PO, AI-assisted)</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Estimates recorded as PO estimates from AI-suggested values – no voting rounds held (see note). Vote columns left empty on purpose. Release PSP = 55 SP; CR-06 = 7 SP</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Session 1 – Release 1.0 baseline (date: 30/10/2026, method: PO estimate from AI suggestion – no voting rounds, facilitator: PO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Round</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Đạt</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Chính</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>Highest/lowest reasoning</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Basis of the estimate</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>Result SP</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>US-01 Register</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr"/>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>US-02 Log in/out</t>
+          <t>US-01 Register</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>–</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>–</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr"/>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>One form; duplicate-email check; client + server validation. Same size as reference 3 (book detail)</t>
+        </is>
+      </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>US-03 Admin creates &amp; locks accounts</t>
+          <t>US-02 Log in/out</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>–</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>–</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr"/>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Session handling + locked-account and generic-error cases; similar to US-01</t>
+        </is>
+      </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>US-04 Server-side access control</t>
+          <t>US-03 Admin creates &amp; locks accounts</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>–</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>–</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr"/>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>List, create, lock/unlock, cannot lock self, session ends on lock; as large as reference 5 (search &amp; filter)</t>
+        </is>
+      </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>NFR-01 Hashing &amp; validation</t>
+          <t>US-04 Server-side access control</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>–</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>–</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr"/>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>One shared server guard, but a 403 check is needed on every /admin route</t>
+        </is>
+      </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>NFR-03 Hosting</t>
+          <t>NFR-01 Hashing &amp; validation</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>–</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>–</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr"/>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>bcrypt library + max-length rules; size of reference 2 (hide book)</t>
+        </is>
+      </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>US-05 Add book</t>
+          <t>NFR-03 Hosting</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>–</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>–</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr"/>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Vercel + Supabase set-up and keep-alive; size of reference 2</t>
+        </is>
+      </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>US-06 Edit book</t>
+          <t>US-05 Add book</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>–</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>–</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr"/>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Most fields of any form + cover upload (JPG/PNG ≤ 2 MB) + boundary checks; reference 5</t>
+        </is>
+      </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>US-07 Hide book</t>
+          <t>US-06 Edit book</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>–</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>–</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr"/>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Reuses the add form; adds not-found and no-change cases</t>
+        </is>
+      </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>US-08 Manage categories</t>
+          <t>US-07 Hide book</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>–</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>–</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr"/>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Reference story (2 SP)</t>
+        </is>
+      </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>US-09 Manage authors</t>
+          <t>US-08 Manage categories</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>–</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>–</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr"/>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Add/rename/remove + unique name + 'in use by N books' rule</t>
+        </is>
+      </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>NFR-02 Seed ≥ 30 books</t>
+          <t>US-09 Manage authors</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>–</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>–</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr"/>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Same pattern as US-08</t>
+        </is>
+      </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>US-10 Book grid</t>
+          <t>NFR-02 Seed ≥ 30 books</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>–</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>–</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr"/>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Seed script that is safe to run twice</t>
+        </is>
+      </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>NFR-04 Responsive UI</t>
+          <t>US-10 Book grid</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>–</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>–</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr"/>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Grid + pagination edge cases (page 0, too large, empty)</t>
+        </is>
+      </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>US-11 Book detail</t>
+          <t>NFR-04 Responsive UI</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>–</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>–</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr"/>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Three breakpoints checked on every page + 44 px tap targets</t>
+        </is>
+      </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>US-12 Search</t>
+          <t>US-11 Book detail</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>–</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>–</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr"/>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Reference story (3 SP); Back keeps page/search/filter</t>
+        </is>
+      </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>US-13 Filter + pagination</t>
+          <t>US-12 Search</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>–</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>–</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr"/>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>One case-insensitive query on title or author; special characters as text</t>
+        </is>
+      </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
+          <t>US-13 Filter + pagination</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Category + price range + search kept in the URL across pages; reference 5</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
           <t>NFR-05 Performance &lt; 2 s</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr"/>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-    </row>
-    <row r="28"/>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>Session 2 – CR-06 impact estimate (before CCB 30/10)</t>
-        </is>
-      </c>
-    </row>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Measure 3 runs on the hosted site; add an index only if needed</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="29"/>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Session 2 – CR-06 impact estimate (30/10/2026, before CCB; same method)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>Round</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>Đạt</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>Chính</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>Reasoning</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>Basis of the estimate</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
         <is>
           <t>Result SP</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>US-24 Store Staff role</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr"/>
-      <c r="F31" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>US-25 Last-updated audit</t>
+          <t>US-24 Store Staff role</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>–</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>–</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr"/>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>New role touches every admin route and screen; server-side checks; as large as US-03</t>
+        </is>
+      </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
+          <t>US-25 Last-updated audit</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Two audit columns + one display line</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
           <t>Rework/regression of F1 (US-03, US-04)</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr"/>
-      <c r="F33" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Rework of existing items; effort is counted in hours (CR-06 C2, C3, C6), not added to PSP</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -4550,12 +4656,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F92"/>
+  <dimension ref="A1:F93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="49" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
@@ -4671,158 +4777,153 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>1.2-draft</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Nguyễn Minh Chính (PO, AI-assisted)</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>SP filled from the PO estimates (planning-poker-log.md v1.1, no voting rounds): PSP = 55 SP, expected velocity 18.3 SP/Sprint; baseline row v1.0 completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>3.2 Milestones (fixed by the brief)</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Milestone</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Date / time (GMT+7)</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Evidence</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>Source</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>M0</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Project start, brief issued</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Fri 23/10</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>[03 §5]</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>M0</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>CR-06 issued by Sponsor</t>
+          <t>Project start, brief issued</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Tue 27/10</t>
+          <t>Fri 23/10</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>CR-06 in Change Log</t>
+          <t>–</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>[CR-06]</t>
+          <t>[03 §5]</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Sprint 1 submission (c1, c2, c3, c0)</t>
+          <t>CR-06 issued by Sponsor</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Thu 29/10 23:59</t>
+          <t>Tue 27/10</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>eLearning upload</t>
+          <t>CR-06 in Change Log</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>[03 §7]</t>
+          <t>[CR-06]</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Review/Retro 1 + CCB for CR-06</t>
+          <t>Sprint 1 submission (c1, c2, c3, c0)</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Fri 30/10</t>
+          <t>Thu 29/10 23:59</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Review slides, CCB decision</t>
+          <t>eLearning upload</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>[03 §5], [CR-06 §5]</t>
+          <t>[03 §7]</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Baseline v1.0 tagged (baseline-v1.0)</t>
+          <t>Review/Retro 1 + CCB for CR-06</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -4832,544 +4933,544 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Git tag</t>
+          <t>Review slides, CCB decision</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>PMP-6</t>
+          <t>[03 §5], [CR-06 §5]</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Sprint 2 submission (c2, c3, c4 CR, c0)</t>
+          <t>Baseline v1.0 tagged (baseline-v1.0)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Thu 05/11 23:59</t>
+          <t>Fri 30/10</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>eLearning upload</t>
+          <t>Git tag</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>[03 §7]</t>
+          <t>PMP-6</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>M6</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Review/Retro 2</t>
+          <t>Sprint 2 submission (c2, c3, c4 CR, c0)</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Fri 06/11</t>
+          <t>Thu 05/11 23:59</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Review slides</t>
+          <t>eLearning upload</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>[03 §5]</t>
+          <t>[03 §7]</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>M7</t>
+          <t>M6</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Release v1.0 tagged + release notes</t>
+          <t>Review/Retro 2</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Thu 12/11</t>
+          <t>Fri 06/11</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Git tag, notes</t>
+          <t>Review slides</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>[03 §6.3]</t>
+          <t>[03 §5]</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>M7</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Sprint 3 submission (c2, c3, c5 UAT, c0)</t>
+          <t>Release v1.0 tagged + release notes</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Thu 12/11 23:59</t>
+          <t>Thu 12/11</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>eLearning upload</t>
+          <t>Git tag, notes</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>[03 §7]</t>
+          <t>[03 §6.3]</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>M9</t>
+          <t>M8</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Review 3 + UAT with customer</t>
+          <t>Sprint 3 submission (c2, c3, c5 UAT, c0)</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Fri 13/11</t>
+          <t>Thu 12/11 23:59</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Signed UAT minutes</t>
+          <t>eLearning upload</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>[03 §6.3]</t>
+          <t>[03 §7]</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>M10</t>
+          <t>M9</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Final submission (c1 Final, c2 Final, c6 Report, c6 Slides, Eval360)</t>
+          <t>Review 3 + UAT with customer</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Sun 15/11 23:59</t>
+          <t>Fri 13/11</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>eLearning upload</t>
+          <t>Signed UAT minutes</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>[03 §7]</t>
+          <t>[03 §6.3]</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Final submission (c1 Final, c2 Final, c6 Report, c6 Slides, Eval360)</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Sun 15/11 23:59</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>eLearning upload</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>[03 §7]</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
           <t>M11</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>Final presentation; site online until end of day</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>Tue 17/11 07:00</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>Live demo</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>[03 §8]</t>
         </is>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>3.3 Sprint plan and leader rotation</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>Sprint</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>Dates</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>Leader</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>Sprint Goal (plan)</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>Increment</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="F27" s="4" t="inlineStr">
         <is>
           <t>PM focus (rubric S4)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>S1 – Plan baseline &amp; F1</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>23/10 – 29/10</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>Hồ Du Tuấn Đạt</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>"Users can register, log in and log out; an administrator can create and lock accounts; non-admins are blocked from admin functions on the server."</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>PMP v1.0</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>S2 – Execution, monitoring &amp; change</t>
+          <t>S1 – Plan baseline &amp; F1</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>30/10 – 05/11</t>
+          <t>23/10 – 29/10</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Nguyễn Minh Chính (PO)</t>
+          <t>Hồ Du Tuấn Đạt</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>"Admins manage books, categories and authors (soft delete), and customers browse 12 books per page, newest first, on any device." (+ CR-06 if approved)</t>
+          <t>"Users can register, log in and log out; an administrator can create and lock accounts; non-admins are blocked from admin functions on the server."</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>F2, F3 (+CR-06)</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>CR + risk/issue</t>
+          <t>PMP v1.0</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>S3 – Complete &amp; acceptance</t>
+          <t>S2 – Execution, monitoring &amp; change</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>06/11 – 12/11</t>
+          <t>30/10 – 05/11</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Hồ Du Tuấn Đạt</t>
+          <t>Nguyễn Minh Chính (PO)</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>"Customers open book details and search/filter by title, author, category and price range together with pagination; Release v1.0 passes UAT."</t>
+          <t>"Admins manage books, categories and authors (soft delete), and customers browse 12 books per page, newest first, on any device." (+ CR-06 if approved)</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>F4, F5</t>
+          <t>F2, F3 (+CR-06)</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>UAT + Release</t>
+          <t>CR + risk/issue</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
+          <t>S3 – Complete &amp; acceptance</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>06/11 – 12/11</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Hồ Du Tuấn Đạt</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>"Customers open book details and search/filter by title, author, category and price range together with pagination; Release v1.0 passes UAT."</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>F4, F5</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>UAT + Release</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
           <t>Closure</t>
         </is>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>13/11 – 17/11</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr">
         <is>
           <t>Final Report, EVM, Lessons Learned, slides, video</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
         <is>
           <t>Release 1.0 online</t>
         </is>
       </c>
-      <c r="F30" s="5" t="inlineStr">
+      <c r="F31" s="5" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
     </row>
-    <row r="31"/>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+    <row r="32"/>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>3.4 Allocation of backlog items to Sprints (plan)</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>Sprint</t>
         </is>
       </c>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>Items</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>SP (plan)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>US-01 Register · US-02 Log in/out · US-03 Admin creates &amp; locks accounts · US-04 Server-side role guard · NFR-01 Password hashing &amp; validation · NFR-03 Hosting/deploy skeleton</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>US-05 Add book · US-06 Edit book · US-07 Hide (soft delete) book · US-08 Manage categories · US-09 Manage authors · NFR-02 Seed ≥30 books · US-10 Book grid 12/page newest first · NFR-04 Responsive UI</t>
+          <t>US-01 Register · US-02 Log in/out · US-03 Admin creates &amp; locks accounts · US-04 Server-side role guard · NFR-01 Password hashing &amp; validation · NFR-03 Hosting/deploy skeleton</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>18</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>S2 (if CR-06 approved, option per CCB)</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>US-24 Store Staff role &amp; permissions · US-25 "Last updated by" audit</t>
+          <t>US-05 Add book · US-06 Edit book · US-07 Hide (soft delete) book · US-08 Manage categories · US-09 Manage authors · NFR-02 Seed ≥30 books · US-10 Book grid 12/page newest first · NFR-04 Responsive UI</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>24</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>S3</t>
+          <t>S2 (if CR-06 approved, option per CCB)</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>US-11 Book detail page (+friendly not-found, Back keeps page) · US-12 Search by title/author · US-13 Filter by category &amp; price range with pagination · NFR-05 List page &lt; 2 s</t>
+          <t>US-24 Store Staff role &amp; permissions · US-25 "Last updated by" audit</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>7 (Option B: US-24 = 5 in S2, US-25 = 2 in S3)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>US-11 Book detail page (+friendly not-found, Back keeps page) · US-12 Search by title/author · US-13 Filter by category &amp; price range with pagination · NFR-05 List page &lt; 2 s</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
           <t>Release 1.0 total</t>
         </is>
       </c>
-      <c r="B38" s="5" t="inlineStr"/>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>PSP = TBD</t>
-        </is>
-      </c>
-    </row>
-    <row r="39"/>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
+      <c r="B39" s="5" t="inlineStr"/>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>PSP = 55 (62 if CR-06 is approved)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40"/>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>3.5 Capacity and expected velocity</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
         <is>
           <t>Sprint</t>
         </is>
       </c>
-      <c r="B41" s="4" t="inlineStr">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>Đạt (h)</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C42" s="4" t="inlineStr">
         <is>
           <t>Chính (h)</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="D42" s="4" t="inlineStr">
         <is>
           <t>Capacity (h)</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
+      <c r="E42" s="4" t="inlineStr">
         <is>
           <t>Source</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>plan/INPUTS.md §2 (plan value, PO 30/10/2026)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
@@ -5387,12 +5488,16 @@
           <t>40</t>
         </is>
       </c>
-      <c r="E43" s="5" t="inlineStr"/>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>plan/INPUTS.md §2 (plan value, PO 30/10/2026)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>S3</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
@@ -5415,114 +5520,105 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
           <t>Release</t>
         </is>
       </c>
-      <c r="B45" s="5" t="inlineStr">
+      <c r="B46" s="5" t="inlineStr">
         <is>
           <t>60</t>
         </is>
       </c>
-      <c r="C45" s="5" t="inlineStr">
+      <c r="C46" s="5" t="inlineStr">
         <is>
           <t>60</t>
         </is>
       </c>
-      <c r="D45" s="5" t="inlineStr">
+      <c r="D46" s="5" t="inlineStr">
         <is>
           <t>120</t>
         </is>
       </c>
-      <c r="E45" s="5" t="inlineStr"/>
-    </row>
-    <row r="46"/>
-    <row r="47">
-      <c r="A47" s="3" t="inlineStr">
+      <c r="E46" s="5" t="inlineStr"/>
+    </row>
+    <row r="47"/>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
         <is>
           <t>3.7 Master schedule (work packages by date)</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="4" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="B48" s="4" t="inlineStr">
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <t>Work package</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="C49" s="4" t="inlineStr">
         <is>
           <t>Start</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
+      <c r="D49" s="4" t="inlineStr">
         <is>
           <t>Due</t>
         </is>
       </c>
-      <c r="E48" s="4" t="inlineStr">
+      <c r="E49" s="4" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="F48" s="4" t="inlineStr">
+      <c r="F49" s="4" t="inlineStr">
         <is>
           <t>Depends on</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
-        <is>
-          <t>Sprint 1 (23–29/10)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>P00</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="inlineStr">
-        <is>
-          <t>Repo, branches, access (GV invited)</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>27/10</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>27/10</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>Đạt</t>
-        </is>
-      </c>
-      <c r="F50" s="5" t="inlineStr">
-        <is>
-          <t>–</t>
+          <t>Sprint 1 (23–29/10)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>P01</t>
+          <t>P00</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Kick-off, roles, working agreement, capacity</t>
+          <t>Repo, branches, access (GV invited)</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
@@ -5532,29 +5628,29 @@
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>28/10</t>
+          <t>27/10</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>P00</t>
+          <t>–</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>P01</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Product Backlog v1.0 (GWT, DoR)</t>
+          <t>Kick-off, roles, working agreement, capacity</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
@@ -5569,61 +5665,61 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>PO</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>P01</t>
+          <t>P00</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>P03</t>
+          <t>P02</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>Planning Poker, Release Plan, BAC</t>
+          <t>Product Backlog v1.0 (GWT, DoR)</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
+          <t>27/10</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
           <t>28/10</t>
         </is>
       </c>
-      <c r="D53" s="5" t="inlineStr">
-        <is>
-          <t>28/10</t>
-        </is>
-      </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>PO + Leader</t>
+          <t>PO</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>P01</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>P03</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>Stack, scaffold, deploy skeleton</t>
+          <t>Planning Poker, Release Plan, BAC</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>27/10</t>
+          <t>28/10</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
@@ -5633,56 +5729,56 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>Đạt</t>
+          <t>PO + Leader</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>P01</t>
+          <t>P02</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>P04</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>Sprint Planning 1 → Jira</t>
+          <t>Stack, scaffold, deploy skeleton</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
+          <t>27/10</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
           <t>28/10</t>
         </is>
       </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>28/10</t>
-        </is>
-      </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>Leader</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>P03</t>
+          <t>P01</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>P06–P07</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>Build F1; F1 test cases</t>
+          <t>Sprint Planning 1 → Jira</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
@@ -5692,34 +5788,34 @@
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>29/10</t>
+          <t>28/10</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Leader</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>P04, P05</t>
+          <t>P03</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P06–P07</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>PMP v1.0 (7 parts)</t>
+          <t>Build F1; F1 test cases</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>27/10</t>
+          <t>28/10</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
@@ -5729,29 +5825,29 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t>Leader + PO</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>P01, P03</t>
+          <t>P04, P05</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>CR-06 Change Log, impact analysis, options</t>
+          <t>PMP v1.0 (7 parts)</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>28/10</t>
+          <t>27/10</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
@@ -5761,29 +5857,29 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t>PO</t>
+          <t>Leader + PO</t>
         </is>
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>P03</t>
+          <t>P01, P03</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P09</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>Daily log, burndown, actual hours</t>
+          <t>CR-06 Change Log, impact analysis, options</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>23/10</t>
+          <t>28/10</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
@@ -5793,36 +5889,36 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t>Leader</t>
+          <t>PO</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>continuous</t>
+          <t>P03</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>Package &amp; submit S1</t>
+          <t>Daily log, burndown, actual hours</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
+          <t>23/10</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
           <t>29/10</t>
         </is>
       </c>
-      <c r="D60" s="5" t="inlineStr">
-        <is>
-          <t>29/10 23:59</t>
-        </is>
-      </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
           <t>Leader</t>
@@ -5830,90 +5926,90 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>above</t>
+          <t>continuous</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>Review/Retro 1 + CCB</t>
+          <t>Package &amp; submit S1</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>30/10</t>
+          <t>29/10</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>30/10</t>
+          <t>29/10 23:59</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>Leader + PO</t>
+          <t>Leader</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>above</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>Sprint 2 (30/10–05/11)</t>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>Review/Retro 1 + CCB</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>30/10</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>30/10</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>Leader + PO</t>
+        </is>
+      </c>
+      <c r="F62" s="5" t="inlineStr">
+        <is>
+          <t>P11</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>P13</t>
-        </is>
-      </c>
-      <c r="B63" s="5" t="inlineStr">
-        <is>
-          <t>Sprint Planning 2 (actual velocity S1)</t>
-        </is>
-      </c>
-      <c r="C63" s="5" t="inlineStr">
-        <is>
-          <t>30/10</t>
-        </is>
-      </c>
-      <c r="D63" s="5" t="inlineStr">
-        <is>
-          <t>30/10</t>
-        </is>
-      </c>
-      <c r="E63" s="5" t="inlineStr">
-        <is>
-          <t>Leader</t>
-        </is>
-      </c>
-      <c r="F63" s="5" t="inlineStr">
-        <is>
-          <t>P12</t>
+          <t>Sprint 2 (30/10–05/11)</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>Update baseline per CCB, tag</t>
+          <t>Sprint Planning 2 (actual velocity S1)</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
@@ -5923,71 +6019,71 @@
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>31/10</t>
+          <t>30/10</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t>PO</t>
+          <t>Leader</t>
         </is>
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>CCB decision</t>
+          <t>P12</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>P15</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>Build F2 (+ seed ≥30 books)</t>
+          <t>Update baseline per CCB, tag</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
+          <t>30/10</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
           <t>31/10</t>
         </is>
       </c>
-      <c r="D65" s="5" t="inlineStr">
-        <is>
-          <t>03/11</t>
-        </is>
-      </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>PO</t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>CCB decision</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P15</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>Build F3</t>
+          <t>Build F2 (+ seed ≥30 books)</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>02/11</t>
+          <t>31/10</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>04/11</t>
+          <t>03/11</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -5997,24 +6093,24 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>P15</t>
+          <t>P13</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>P17</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>Build CR-06 (if approved)</t>
+          <t>Build F3</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>01/11</t>
+          <t>02/11</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
@@ -6029,29 +6125,29 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>P15</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>P18</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>Test cases F2, F3, CR-06 + regression F1</t>
+          <t>Build CR-06 (if approved)</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>03/11</t>
+          <t>01/11</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>05/11</t>
+          <t>04/11</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -6061,24 +6157,24 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>P15–P17</t>
+          <t>P14</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>P19</t>
+          <t>P18</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>Weekly Status, risk &amp; issue log</t>
+          <t>Test cases F2, F3, CR-06 + regression F1</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>30/10</t>
+          <t>03/11</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
@@ -6088,29 +6184,29 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t>Leader</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>continuous</t>
+          <t>P15–P17</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>P20</t>
+          <t>P19</t>
         </is>
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>c4 Change Request form</t>
+          <t>Weekly Status, risk &amp; issue log</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>31/10</t>
+          <t>30/10</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
@@ -6120,66 +6216,66 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t>PO</t>
+          <t>Leader</t>
         </is>
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>continuous</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>P21</t>
+          <t>P20</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>Package &amp; submit S2</t>
+          <t>c4 Change Request form</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
+          <t>31/10</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
           <t>05/11</t>
         </is>
       </c>
-      <c r="D71" s="5" t="inlineStr">
-        <is>
-          <t>05/11 23:59</t>
-        </is>
-      </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t>Leader</t>
+          <t>PO</t>
         </is>
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>above</t>
+          <t>P14</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>P22</t>
+          <t>P21</t>
         </is>
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>Review/Retro 2</t>
+          <t>Package &amp; submit S2</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>06/11</t>
+          <t>05/11</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>06/11</t>
+          <t>05/11 23:59</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -6189,102 +6285,102 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>P21</t>
+          <t>above</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>Sprint 3 (06–12/11)</t>
+          <t>P22</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>Review/Retro 2</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>06/11</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>06/11</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>Leader</t>
+        </is>
+      </c>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>P21</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>P23</t>
-        </is>
-      </c>
-      <c r="B74" s="5" t="inlineStr">
-        <is>
-          <t>Sprint Planning 3 (actual velocity S2)</t>
-        </is>
-      </c>
-      <c r="C74" s="5" t="inlineStr">
-        <is>
-          <t>06/11</t>
-        </is>
-      </c>
-      <c r="D74" s="5" t="inlineStr">
-        <is>
-          <t>06/11</t>
-        </is>
-      </c>
-      <c r="E74" s="5" t="inlineStr">
-        <is>
-          <t>Leader</t>
-        </is>
-      </c>
-      <c r="F74" s="5" t="inlineStr">
-        <is>
-          <t>P22</t>
+          <t>Sprint 3 (06–12/11)</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>P24–P25</t>
+          <t>P23</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>Build F4, F5</t>
+          <t>Sprint Planning 3 (actual velocity S2)</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>07/11</t>
+          <t>06/11</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>10/11</t>
+          <t>06/11</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Leader</t>
         </is>
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>P23</t>
+          <t>P22</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>P26</t>
+          <t>P24–P25</t>
         </is>
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>Tests F4, F5, regression F1–F3, performance</t>
+          <t>Build F4, F5</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
+          <t>07/11</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr">
+        <is>
           <t>10/11</t>
         </is>
       </c>
-      <c r="D76" s="5" t="inlineStr">
-        <is>
-          <t>11/11</t>
-        </is>
-      </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
           <t>Both</t>
@@ -6292,56 +6388,56 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>P24, P25</t>
+          <t>P23</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>P27</t>
+          <t>P26</t>
         </is>
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>Release v1.0: merge to main, tag, notes</t>
+          <t>Tests F4, F5, regression F1–F3, performance</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
+          <t>10/11</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
           <t>11/11</t>
         </is>
       </c>
-      <c r="D77" s="5" t="inlineStr">
-        <is>
-          <t>12/11</t>
-        </is>
-      </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t>Leader</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>P26</t>
+          <t>P24, P25</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>P28</t>
+          <t>P27</t>
         </is>
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>UAT script (all ACs)</t>
+          <t>Release v1.0: merge to main, tag, notes</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>10/11</t>
+          <t>11/11</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
@@ -6351,7 +6447,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t>PO</t>
+          <t>Leader</t>
         </is>
       </c>
       <c r="F78" s="5" t="inlineStr">
@@ -6363,17 +6459,17 @@
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>P29</t>
+          <t>P28</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>Monitoring + draft EVM</t>
+          <t>UAT script (all ACs)</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>06/11</t>
+          <t>10/11</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
@@ -6383,36 +6479,36 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Leader</t>
+          <t>PO</t>
         </is>
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>continuous</t>
+          <t>P26</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>P30</t>
+          <t>P29</t>
         </is>
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>Package &amp; submit S3</t>
+          <t>Monitoring + draft EVM</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
+          <t>06/11</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
           <t>12/11</t>
         </is>
       </c>
-      <c r="D80" s="5" t="inlineStr">
-        <is>
-          <t>12/11 23:59</t>
-        </is>
-      </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
           <t>Leader</t>
@@ -6420,90 +6516,90 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>above</t>
+          <t>continuous</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>P31</t>
+          <t>P30</t>
         </is>
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>Review 3 + UAT + minutes</t>
+          <t>Package &amp; submit S3</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>13/11</t>
+          <t>12/11</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>13/11</t>
+          <t>12/11 23:59</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t>Leader + PO</t>
+          <t>Leader</t>
         </is>
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>P30</t>
+          <t>above</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>Closure (13–17/11)</t>
+          <t>P31</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>Review 3 + UAT + minutes</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>13/11</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>13/11</t>
+        </is>
+      </c>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>Leader + PO</t>
+        </is>
+      </c>
+      <c r="F82" s="5" t="inlineStr">
+        <is>
+          <t>P30</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>P32</t>
-        </is>
-      </c>
-      <c r="B83" s="5" t="inlineStr">
-        <is>
-          <t>Final hosting, demo accounts, closure data</t>
-        </is>
-      </c>
-      <c r="C83" s="5" t="inlineStr">
-        <is>
-          <t>13/11</t>
-        </is>
-      </c>
-      <c r="D83" s="5" t="inlineStr">
-        <is>
-          <t>14/11</t>
-        </is>
-      </c>
-      <c r="E83" s="5" t="inlineStr">
-        <is>
-          <t>Đạt</t>
-        </is>
-      </c>
-      <c r="F83" s="5" t="inlineStr">
-        <is>
-          <t>P31</t>
+          <t>Closure (13–17/11)</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>P33</t>
+          <t>P32</t>
         </is>
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>Final Report, EVM, Lessons Learned, PMP/Workbook Final</t>
+          <t>Final hosting, demo accounts, closure data</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
@@ -6513,34 +6609,34 @@
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>15/11</t>
+          <t>14/11</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>P31, P32</t>
+          <t>P31</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>P34</t>
+          <t>P33</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>Slides + demo video ≤ 3 min</t>
+          <t>Final Report, EVM, Lessons Learned, PMP/Workbook Final</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>14/11</t>
+          <t>13/11</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
@@ -6555,31 +6651,31 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>P33</t>
+          <t>P31, P32</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>P35</t>
+          <t>P34</t>
         </is>
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>Final submission + Eval360 each</t>
+          <t>Slides + demo video ≤ 3 min</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
+          <t>14/11</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
           <t>15/11</t>
         </is>
       </c>
-      <c r="D86" s="5" t="inlineStr">
-        <is>
-          <t>15/11 23:59</t>
-        </is>
-      </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
           <t>Both</t>
@@ -6587,141 +6683,173 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>P33, P34</t>
+          <t>P33</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
+          <t>P35</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>Final submission + Eval360 each</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>15/11</t>
+        </is>
+      </c>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>15/11 23:59</t>
+        </is>
+      </c>
+      <c r="E87" s="5" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F87" s="5" t="inlineStr">
+        <is>
+          <t>P33, P34</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="5" t="inlineStr">
+        <is>
           <t>P36</t>
         </is>
       </c>
-      <c r="B87" s="5" t="inlineStr">
+      <c r="B88" s="5" t="inlineStr">
         <is>
           <t>Final presentation</t>
         </is>
       </c>
-      <c r="C87" s="5" t="inlineStr">
+      <c r="C88" s="5" t="inlineStr">
         <is>
           <t>16/11</t>
         </is>
       </c>
-      <c r="D87" s="5" t="inlineStr">
+      <c r="D88" s="5" t="inlineStr">
         <is>
           <t>17/11 07:00</t>
         </is>
       </c>
-      <c r="E87" s="5" t="inlineStr">
+      <c r="E88" s="5" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="F87" s="5" t="inlineStr">
+      <c r="F88" s="5" t="inlineStr">
         <is>
           <t>P35</t>
         </is>
       </c>
     </row>
-    <row r="88"/>
-    <row r="89">
-      <c r="A89" s="3" t="inlineStr">
+    <row r="89"/>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
         <is>
           <t>3.8 Baseline and change history of this plan</t>
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="4" t="inlineStr">
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr">
         <is>
           <t>Baseline</t>
         </is>
       </c>
-      <c r="B90" s="4" t="inlineStr">
+      <c r="B91" s="4" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C90" s="4" t="inlineStr">
+      <c r="C91" s="4" t="inlineStr">
         <is>
           <t>Trigger</t>
         </is>
       </c>
-      <c r="D90" s="4" t="inlineStr">
+      <c r="D91" s="4" t="inlineStr">
         <is>
           <t>PSP</t>
         </is>
       </c>
-      <c r="E90" s="4" t="inlineStr">
+      <c r="E91" s="4" t="inlineStr">
         <is>
           <t>BAC</t>
         </is>
       </c>
-      <c r="F90" s="4" t="inlineStr">
+      <c r="F91" s="4" t="inlineStr">
         <is>
           <t>Tag</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="5" t="inlineStr">
-        <is>
-          <t>Baseline v1.0</t>
-        </is>
-      </c>
-      <c r="B91" s="5" t="inlineStr">
-        <is>
-          <t>30/10/2026</t>
-        </is>
-      </c>
-      <c r="C91" s="5" t="inlineStr">
-        <is>
-          <t>Sprint 1 submission</t>
-        </is>
-      </c>
-      <c r="D91" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E91" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F91" s="5" t="inlineStr">
-        <is>
-          <t>baseline-v1.0</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
+          <t>Baseline v1.0</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>Sprint 1 submission</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>55 SP</t>
+        </is>
+      </c>
+      <c r="E92" s="5" t="inlineStr">
+        <is>
+          <t>24,000,000 VND</t>
+        </is>
+      </c>
+      <c r="F92" s="5" t="inlineStr">
+        <is>
+          <t>baseline-v1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="5" t="inlineStr">
+        <is>
           <t>Rebaseline v1.1</t>
         </is>
       </c>
-      <c r="B92" s="5" t="inlineStr">
+      <c r="B93" s="5" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="C92" s="5" t="inlineStr">
+      <c r="C93" s="5" t="inlineStr">
         <is>
           <t>CCB decision on CR-06 (if Approve)</t>
         </is>
       </c>
-      <c r="D92" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E92" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F92" s="5" t="inlineStr">
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>62 SP (proposed)</t>
+        </is>
+      </c>
+      <c r="E93" s="5" t="inlineStr">
+        <is>
+          <t>per CCB decision</t>
+        </is>
+      </c>
+      <c r="F93" s="5" t="inlineStr">
         <is>
           <t>baseline-v1.1</t>
         </is>

</xml_diff>